<commit_message>
UI Overhaul: Added 3D animations, background slideshow, and updated system identity to Shah Nawaz Hussain
</commit_message>
<xml_diff>
--- a/System_Users.xlsx
+++ b/System_Users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -442,24 +442,58 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>SHAHIL</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SHAHIL</v>
+      </c>
+      <c r="C3" t="str">
+        <v>shahil</v>
+      </c>
+      <c r="D3" t="str">
+        <v>analyst</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Shahil@123</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
         <v>ANSHU</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B4" t="str">
         <v>ANSHU</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C4" t="str">
         <v>anshu</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D4" t="str">
         <v>clerk</v>
       </c>
-      <c r="E3" t="str">
-        <v>123</v>
+      <c r="E4" t="str">
+        <v>Shahil@123</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>JP</v>
+      </c>
+      <c r="B5" t="str">
+        <v>JP</v>
+      </c>
+      <c r="C5" t="str">
+        <v>jp</v>
+      </c>
+      <c r="D5" t="str">
+        <v>analyst</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Shahil@123</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: fix edit modal layout and update system users
</commit_message>
<xml_diff>
--- a/System_Users.xlsx
+++ b/System_Users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -491,9 +491,43 @@
         <v>Shahil@123</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ASA</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ASA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>asa</v>
+      </c>
+      <c r="D6" t="str">
+        <v>viewer</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Shahil@123</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Test Clerk</v>
+      </c>
+      <c r="D7" t="str">
+        <v>clerk</v>
+      </c>
+      <c r="E7" t="str">
+        <v>123Pass@123</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: mobile card layout for records table + fix useCallback hooks violation + sticky Edit Modal footer
</commit_message>
<xml_diff>
--- a/System_Users.xlsx
+++ b/System_Users.xlsx
@@ -476,16 +476,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>JP</v>
+        <v>ASA</v>
       </c>
       <c r="B5" t="str">
-        <v>JP</v>
+        <v>ASA</v>
       </c>
       <c r="C5" t="str">
-        <v>jp</v>
+        <v>asa</v>
       </c>
       <c r="D5" t="str">
-        <v>analyst</v>
+        <v>viewer</v>
       </c>
       <c r="E5" t="str">
         <v>Shahil@123</v>
@@ -493,36 +493,36 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ASA</v>
+        <v>TEST</v>
       </c>
       <c r="B6" t="str">
-        <v>ASA</v>
+        <v>TEST</v>
       </c>
       <c r="C6" t="str">
-        <v>asa</v>
+        <v>Test Clerk</v>
       </c>
       <c r="D6" t="str">
-        <v>viewer</v>
+        <v>clerk</v>
       </c>
       <c r="E6" t="str">
-        <v>Shahil@123</v>
+        <v>123Pass@123</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TEST</v>
+        <v>HUSSS</v>
       </c>
       <c r="B7" t="str">
-        <v>TEST</v>
+        <v>HUSSS</v>
       </c>
       <c r="C7" t="str">
-        <v>Test Clerk</v>
+        <v>haush</v>
       </c>
       <c r="D7" t="str">
-        <v>clerk</v>
+        <v>viewer</v>
       </c>
       <c r="E7" t="str">
-        <v>123Pass@123</v>
+        <v>Shahil@123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>